<commit_message>
Add Others field in the Transaction Production Calculation and made into the calculation
</commit_message>
<xml_diff>
--- a/Purchase invoice Calculation.xlsx
+++ b/Purchase invoice Calculation.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="29">
   <si>
     <t>COST FACTOR CALCULATION FOR THE PRODUCT BASED ON HEAD ON HEAD LESS</t>
   </si>
@@ -62,14 +62,62 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t>RATE CALCULATION FOR EACH SLAB</t>
+  </si>
+  <si>
+    <t>IT MAY BE ANYTHING @70, @72, @75</t>
+  </si>
+  <si>
+    <t>HEAD ON</t>
+  </si>
+  <si>
+    <t>SLAB</t>
+  </si>
+  <si>
+    <t>VALUE</t>
+  </si>
+  <si>
+    <t>U - 15</t>
+  </si>
+  <si>
+    <t>20 - 30</t>
+  </si>
+  <si>
+    <t>30 - 40</t>
+  </si>
+  <si>
+    <t>10 -- 20</t>
+  </si>
+  <si>
+    <t>MULTIPLY SLAB X VALUE</t>
+  </si>
+  <si>
+    <t>MANUAL VALUE</t>
+  </si>
+  <si>
+    <t>DOLLAR RATE IT CAN BE ANYTHING (FOR EG.., 70, 72, 75)</t>
+  </si>
+  <si>
+    <t>IN THIS WE TAKE $ 70</t>
+  </si>
+  <si>
+    <t>TOTAL VALUE FOR DOLLAR</t>
+  </si>
+  <si>
+    <t>TOTAL DOLLAR VALUE DIVIDE BY NET WEIGHT IS GIVING PER KG DOLLAR VALUE</t>
+  </si>
+  <si>
+    <t>NET WEIGHT</t>
+  </si>
+  <si>
+    <t>MULTIPLY TOTAL WITH MANUAL VALUE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,8 +155,55 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -135,8 +230,25 @@
         <fgColor rgb="FFA5A5A5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -174,27 +286,62 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="3"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="4"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="5" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="5">
+  <cellStyles count="6">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
     <cellStyle name="Calculation" xfId="3" builtinId="22"/>
     <cellStyle name="Check Cell" xfId="4" builtinId="23"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="5" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -473,17 +620,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="68.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.6640625" customWidth="1"/>
-    <col min="5" max="5" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5546875" customWidth="1"/>
+    <col min="5" max="5" width="26.21875" customWidth="1"/>
+    <col min="6" max="6" width="48.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B1" t="s">
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
     </row>
@@ -583,7 +731,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="17" spans="3:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
@@ -592,10 +740,161 @@
         <v>15218.999999999998</v>
       </c>
     </row>
-    <row r="18" spans="3:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C22" t="s">
+    <row r="18" spans="2:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="4" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B24" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="9">
+        <v>10</v>
+      </c>
+      <c r="D24" s="9">
+        <v>10.5</v>
+      </c>
+      <c r="E24" s="9">
+        <f>C24*D24</f>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B25" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="9">
+        <v>17</v>
+      </c>
+      <c r="D25" s="9">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="E25" s="9">
+        <f>C25*D25</f>
+        <v>166.60000000000002</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="9">
+        <v>31</v>
+      </c>
+      <c r="D26" s="9">
+        <v>7</v>
+      </c>
+      <c r="E26" s="9">
+        <f>C26*D26</f>
+        <v>217</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B27" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="9">
+        <v>5</v>
+      </c>
+      <c r="D27" s="9">
+        <v>5.8</v>
+      </c>
+      <c r="E27" s="9">
+        <f>C27*D27</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" s="16">
+        <f>E24+E25+E26+E27</f>
+        <v>517.6</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="D31" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="E31" s="17">
+        <v>1.4</v>
+      </c>
+      <c r="F31" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="F32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="4:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="D33" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E33" s="15">
+        <f>E29*E31</f>
+        <v>724.64</v>
+      </c>
+      <c r="F33" s="14">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35" spans="4:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="36" spans="4:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E36" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F36" s="12">
+        <f>E33*F33</f>
+        <v>50724.799999999996</v>
+      </c>
+    </row>
+    <row r="37" spans="4:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="38" spans="4:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E38" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F38" s="12">
+        <v>90.09</v>
+      </c>
+    </row>
+    <row r="39" spans="4:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="4:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="E40" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F40" s="13">
+        <f>F36/F38</f>
+        <v>563.04584304584296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add R button in the Raw Material Invoice Form
</commit_message>
<xml_diff>
--- a/Purchase invoice Calculation.xlsx
+++ b/Purchase invoice Calculation.xlsx
@@ -74,9 +74,6 @@
     <t>SLAB</t>
   </si>
   <si>
-    <t>VALUE</t>
-  </si>
-  <si>
     <t>U - 15</t>
   </si>
   <si>
@@ -92,12 +89,6 @@
     <t>MULTIPLY SLAB X VALUE</t>
   </si>
   <si>
-    <t>MANUAL VALUE</t>
-  </si>
-  <si>
-    <t>DOLLAR RATE IT CAN BE ANYTHING (FOR EG.., 70, 72, 75)</t>
-  </si>
-  <si>
     <t>IN THIS WE TAKE $ 70</t>
   </si>
   <si>
@@ -111,6 +102,15 @@
   </si>
   <si>
     <t>MULTIPLY TOTAL WITH MANUAL VALUE</t>
+  </si>
+  <si>
+    <t>VALUE (MANUAL VALUE NOT FIXED)</t>
+  </si>
+  <si>
+    <t>DOLLAR RATE IT CAN BE ANYTHING (FOR EG.., 70, 72, 75)(MANUAL VALUE NOT FIXED)</t>
+  </si>
+  <si>
+    <t>(MANUAL VALUE NOT FIXED)</t>
   </si>
 </sst>
 </file>
@@ -310,7 +310,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="3"/>
@@ -335,6 +335,9 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -751,18 +754,18 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B22" s="7" t="s">
         <v>14</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="7" t="s">
-        <v>16</v>
+      <c r="D22" s="18" t="s">
+        <v>26</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
@@ -773,7 +776,7 @@
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C24" s="9">
         <v>10</v>
@@ -788,7 +791,7 @@
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C25" s="9">
         <v>17</v>
@@ -803,7 +806,7 @@
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C26" s="9">
         <v>31</v>
@@ -818,7 +821,7 @@
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C27" s="9">
         <v>5</v>
@@ -840,25 +843,25 @@
         <v>517.6</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D31" s="11" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E31" s="17">
         <v>1.4</v>
       </c>
-      <c r="F31" t="s">
-        <v>23</v>
+      <c r="F31" s="11" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="F32" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="33" spans="4:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D33" s="11" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E33" s="15">
         <f>E29*E31</f>
@@ -871,7 +874,7 @@
     <row r="35" spans="4:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="36" spans="4:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E36" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F36" s="12">
         <f>E33*F33</f>
@@ -881,7 +884,7 @@
     <row r="37" spans="4:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="38" spans="4:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E38" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F38" s="12">
         <v>90.09</v>
@@ -890,7 +893,7 @@
     <row r="39" spans="4:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
     <row r="40" spans="4:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="E40" s="11" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F40" s="13">
         <f>F36/F38</f>

</xml_diff>

<commit_message>
Documentation the new feature incentive calculation
</commit_message>
<xml_diff>
--- a/Purchase invoice Calculation.xlsx
+++ b/Purchase invoice Calculation.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
   <si>
     <t>COST FACTOR CALCULATION FOR THE PRODUCT BASED ON HEAD ON HEAD LESS</t>
   </si>
@@ -111,13 +111,22 @@
   </si>
   <si>
     <t>(MANUAL VALUE NOT FIXED)</t>
+  </si>
+  <si>
+    <t>TOTAL DOLLAR VALUE WITH 5 %</t>
+  </si>
+  <si>
+    <t>ADD TAX CONVERTED VALUES + TOTAL VALUE FOR DOLLAR</t>
+  </si>
+  <si>
+    <t>IN THIS THEY GIVE INCENTIVE FOR THE SUPPLIER IT CAN BE ANYTHING (IN THIS I GIVE 5 PERCENTAGE)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,8 +211,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFF00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -244,6 +261,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -310,7 +333,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="3"/>
@@ -337,6 +360,18 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="4" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -623,7 +658,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="68.21875" bestFit="1" customWidth="1"/>
@@ -631,6 +666,9 @@
     <col min="4" max="4" width="14.5546875" customWidth="1"/>
     <col min="5" max="5" width="26.21875" customWidth="1"/>
     <col min="6" max="6" width="48.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.88671875" customWidth="1"/>
+    <col min="9" max="9" width="14.21875" customWidth="1"/>
+    <col min="11" max="11" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -859,7 +897,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="4:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="4:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D33" s="11" t="s">
         <v>25</v>
       </c>
@@ -871,8 +909,8 @@
         <v>70</v>
       </c>
     </row>
-    <row r="35" spans="4:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="36" spans="4:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="4:12" ht="43.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="36" spans="4:12" ht="63.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E36" s="3" t="s">
         <v>22</v>
       </c>
@@ -880,9 +918,29 @@
         <f>E33*F33</f>
         <v>50724.799999999996</v>
       </c>
-    </row>
-    <row r="37" spans="4:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="38" spans="4:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G36" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="H36" s="20">
+        <v>0.05</v>
+      </c>
+      <c r="I36" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="J36" s="21">
+        <f>F36*H36</f>
+        <v>2536.2399999999998</v>
+      </c>
+      <c r="K36" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="L36" s="22">
+        <f>F36+J36</f>
+        <v>53261.039999999994</v>
+      </c>
+    </row>
+    <row r="37" spans="4:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="38" spans="4:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E38" s="3" t="s">
         <v>24</v>
       </c>
@@ -890,14 +948,14 @@
         <v>90.09</v>
       </c>
     </row>
-    <row r="39" spans="4:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="40" spans="4:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="4:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="4:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="E40" s="11" t="s">
         <v>23</v>
       </c>
       <c r="F40" s="13">
-        <f>F36/F38</f>
-        <v>563.04584304584296</v>
+        <f>L36/F38</f>
+        <v>591.19813519813511</v>
       </c>
     </row>
   </sheetData>

</xml_diff>